<commit_message>
Populate MWG v3 segment history and assumptions for TGDD DMX BHX
</commit_message>
<xml_diff>
--- a/MWG_valuation_model_v3.xlsx
+++ b/MWG_valuation_model_v3.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPO_DMX" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Input_Notes" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -823,7 +824,9 @@
           <t>An Khang</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>2500</v>
+      </c>
       <c r="C2" s="2">
         <f>B2*(1+Micro_Drivers!C10)</f>
         <v/>
@@ -862,7 +865,9 @@
           <t>AVAKids / specialty retail</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="n">
+        <v>3500</v>
+      </c>
       <c r="C3" s="2">
         <f>B3*(1+Micro_Drivers!C10)</f>
         <v/>
@@ -901,7 +906,9 @@
           <t>Other / online / services</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="n">
+        <v>33000</v>
+      </c>
       <c r="C4" s="2">
         <f>B4*(1+Micro_Drivers!C10)</f>
         <v/>
@@ -2462,6 +2469,127 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Mục</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Cách em input hiện tại</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Mức độ tin cậy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TGDD/ĐMX/BHX revenue history</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ước lượng dựa trên quy mô tương đối của các mảng và tổng doanh thu MWG, dùng để model chạy chi tiết ngay.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Medium-low until official segment disclosures are keyed in</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BHX margin history</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Đặt đường cong từ lỗ sang gần hòa vốn/lãi nhẹ để phản ánh turnaround.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DMX market share</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Assumption leader position ~50%+ in modern CE retail.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Medium-low</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Other revenue</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Residual = consolidated less core segments.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mục tiêu</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cho anh có model chi tiết chạy được ngay; vòng sau nên thay bằng số từ annual report/presentation/BCTC note nếu trích được sạch.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2518,7 +2646,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>68000</v>
+        <v>70000</v>
       </c>
       <c r="C2" s="6" t="n">
         <v>68000</v>
@@ -2674,7 +2802,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>0.048</v>
+        <v>0.05</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>0.053</v>
@@ -2882,7 +3010,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>0.6</v>
@@ -2908,7 +3036,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>0.8</v>
@@ -3372,12 +3500,26 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>122958</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>133405</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>118280</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>134341</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Revenue est/placeholder, 2025 raised above 2024 based on 2025 audited existence + recovery cycle</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3385,12 +3527,26 @@
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="n">
+        <v>26757</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>28800</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>23600</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>28800</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>33000</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Gross profit placeholder refined</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3398,12 +3554,26 @@
           <t>EBIT</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="n">
+        <v>6600</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>6200</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>4700</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>6200</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>EBIT placeholder refined</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3411,12 +3581,26 @@
           <t>NPAT</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="n">
+        <v>4900</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>4100</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>3600</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>4700</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>NPAT placeholder refined</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3424,12 +3608,26 @@
           <t>Operating CF</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="n">
+        <v>8500</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>9800</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Operating CF placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3437,12 +3635,26 @@
           <t>Capex</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="n">
+        <v>2200</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Capex placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3450,12 +3662,26 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="n">
+        <v>14500</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>13000</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>17000</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Cash placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3463,12 +3689,26 @@
           <t>Debt</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="n">
+        <v>21500</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>19500</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>21000</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>24000</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Debt placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3476,12 +3716,26 @@
           <t>Net debt</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>6500</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Net debt placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3489,12 +3743,26 @@
           <t>Total assets</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="n">
+        <v>59000</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>62000</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>65000</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>72000</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Assets placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3502,12 +3770,26 @@
           <t>Equity</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="n">
+        <v>22000</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>24500</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>27500</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Equity placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -3601,12 +3883,26 @@
           <t>TGDD revenue</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>26000</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>26500</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>25500</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>26000</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>TGDD revenue - placeholder conservative, mature/saturated</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3614,12 +3910,26 @@
           <t>TGDD store count</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>880</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>850</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>820</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>TGDD store count placeholder, optimization downtrend</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3627,12 +3937,26 @@
           <t>TGDD revenue/store</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>TGDD revenue/store = revenue/count approx</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3640,12 +3964,26 @@
           <t>DMX revenue</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="n">
+        <v>52000</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>56000</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>56000</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>62000</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>ĐMX revenue placeholder, major earnings engine</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3653,12 +3991,26 @@
           <t>DMX store count</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1850</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>ĐMX store count placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3666,12 +4018,26 @@
           <t>DMX revenue/store</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>ĐMX revenue/store approx</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3679,12 +4045,26 @@
           <t>DMX market share</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>ĐMX market share placeholder based on leading position</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3692,12 +4072,26 @@
           <t>BHX revenue</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="n">
+        <v>28000</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>31500</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>49000</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>BHX revenue placeholder, fast growth</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3705,12 +4099,26 @@
           <t>BHX store count</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1700</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1750</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>BHX store count placeholder after restructuring and reopening growth</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3718,12 +4126,26 @@
           <t>BHX revenue/store</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>BHX revenue/store approx</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3731,12 +4153,26 @@
           <t>BHX EBIT margin</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>BHX EBIT margin path placeholder: loss to near breakeven/profit</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3744,12 +4180,26 @@
           <t>BHX market share</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>BHX market share placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3757,12 +4207,26 @@
           <t>Other revenue</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="n">
+        <v>44958</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>50905</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>42780</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>38841</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>39000</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Other revenue residual from consolidated less core segments</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4140,7 +4604,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>Segment_Historical!C2</f>
+        <f>Segment_Historical!F3</f>
         <v/>
       </c>
       <c r="C2" s="2">
@@ -4176,7 +4640,7 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>Segment_Historical!C3</f>
+        <f>Segment_Historical!F4</f>
         <v/>
       </c>
       <c r="C3" s="2">
@@ -4212,7 +4676,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>Segment_Historical!C4</f>
+        <f>Segment_Historical!F2</f>
         <v/>
       </c>
       <c r="C4" s="2">
@@ -4403,7 +4867,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>Segment_Historical!C5</f>
+        <f>Segment_Historical!F6</f>
         <v/>
       </c>
       <c r="C2" s="2">
@@ -4439,7 +4903,7 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>Segment_Historical!C8</f>
+        <f>Segment_Historical!F8</f>
         <v/>
       </c>
       <c r="C3" s="2">
@@ -4471,7 +4935,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>Segment_Historical!C7</f>
+        <f>Segment_Historical!F7</f>
         <v/>
       </c>
       <c r="C4" s="2">
@@ -4503,7 +4967,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>Segment_Historical!C6</f>
+        <f>Segment_Historical!F5</f>
         <v/>
       </c>
       <c r="C5" s="2">
@@ -4694,7 +5158,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>Segment_Historical!C10</f>
+        <f>Segment_Historical!F10</f>
         <v/>
       </c>
       <c r="C2" s="2">
@@ -4761,7 +5225,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>Segment_Historical!C11</f>
+        <f>Segment_Historical!F11</f>
         <v/>
       </c>
       <c r="C4" s="2">
@@ -4824,7 +5288,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>Segment_Historical!C9</f>
+        <f>Segment_Historical!F9</f>
         <v/>
       </c>
       <c r="C6" s="2">
@@ -4885,7 +5349,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>Segment_Historical!C12</f>
+        <f>Segment_Historical!F12</f>
         <v/>
       </c>
       <c r="C8" s="2">
@@ -4949,7 +5413,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <f>Segment_Historical!C13</f>
+        <f>Segment_Historical!F13</f>
         <v/>
       </c>
       <c r="C10" s="2">

</xml_diff>